<commit_message>
Enhance Excel file manipulation by adding formulas, styling, and borders
</commit_message>
<xml_diff>
--- a/Book/chapter14/myExcelFile.xlsx
+++ b/Book/chapter14/myExcelFile.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,16 +31,55 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="003F27F5"/>
+      <sz val="32"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="mediumGray">
+        <fgColor rgb="00BBF527"/>
+        <bgColor rgb="00F5275E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <gradientFill type="linear">
+        <stop position="0">
+          <color rgb="00000000"/>
+        </stop>
+        <stop position="1">
+          <color rgb="00FFFFFF"/>
+        </stop>
+      </gradientFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000FF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,13 +87,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="dotted">
+        <color rgb="00000000"/>
+      </left>
+      <right style="dotted">
+        <color rgb="00000000"/>
+      </right>
+      <top style="dashed">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,50 +513,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Names</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Ages</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Overdue</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Dates</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Due Soon</t>
+        </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46138.38308118264</v>
+        <v>46138.44337213237</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>On Time</t>
+        </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.38308118278</v>
+        <v>46138.44337213253</v>
       </c>
     </row>
     <row r="4">
@@ -502,7 +573,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.38308118286</v>
+        <v>46138.44337213263</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +586,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.38308118292</v>
+        <v>46138.44337213269</v>
       </c>
     </row>
     <row r="6">
@@ -528,7 +599,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.38308118298</v>
+        <v>46138.44337213277</v>
       </c>
     </row>
     <row r="7">
@@ -541,7 +612,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.38308118304</v>
+        <v>46138.44337213284</v>
       </c>
     </row>
     <row r="8">
@@ -554,7 +625,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.3830811831</v>
+        <v>46138.44337213292</v>
       </c>
     </row>
     <row r="9">
@@ -567,7 +638,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.38308118316</v>
+        <v>46138.44337213298</v>
       </c>
     </row>
     <row r="10">
@@ -580,7 +651,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.38308118322</v>
+        <v>46138.44337213306</v>
       </c>
     </row>
     <row r="11">
@@ -593,7 +664,31 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.38308118327</v>
+        <v>46138.44337213312</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12">
+        <f>SUM(B2:B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13">
+        <f>AVERAGE(B2:B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14">
+        <f>IF(A1="Carlos",True,False)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7">
+        <f>VLOOKUP("c",A1:C11,2,FALSE)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -650,7 +745,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46138.38308118264</v>
+        <v>46138.44337213237</v>
       </c>
     </row>
     <row r="3">
@@ -663,7 +758,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.38308118278</v>
+        <v>46138.44337213253</v>
       </c>
     </row>
     <row r="4">
@@ -676,7 +771,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.38308118286</v>
+        <v>46138.44337213263</v>
       </c>
     </row>
     <row r="5">
@@ -689,7 +784,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.38308118292</v>
+        <v>46138.44337213269</v>
       </c>
     </row>
     <row r="6">
@@ -702,7 +797,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.38308118298</v>
+        <v>46138.44337213277</v>
       </c>
     </row>
     <row r="7">
@@ -715,7 +810,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.38308118304</v>
+        <v>46138.44337213284</v>
       </c>
     </row>
     <row r="8">
@@ -728,7 +823,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.3830811831</v>
+        <v>46138.44337213292</v>
       </c>
     </row>
     <row r="9">
@@ -741,7 +836,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.38308118316</v>
+        <v>46138.44337213298</v>
       </c>
     </row>
     <row r="10">
@@ -754,7 +849,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.38308118322</v>
+        <v>46138.44337213306</v>
       </c>
     </row>
     <row r="11">
@@ -767,7 +862,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.38308118327</v>
+        <v>46138.44337213312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance Excel file manipulation by adding cell alignment, adjusting row and column dimensions, and implementing cell merging functionality
</commit_message>
<xml_diff>
--- a/Book/chapter14/myExcelFile.xlsx
+++ b/Book/chapter14/myExcelFile.xlsx
@@ -79,27 +79,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="dotted">
-        <color rgb="00000000"/>
-      </left>
-      <right style="dotted">
-        <color rgb="00000000"/>
-      </right>
-      <top style="dashed">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="dashed">
-        <color rgb="00000000"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -121,7 +107,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -514,17 +502,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col hidden="1" width="13" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Names</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Overdue</t>
+          <t>Different value</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
@@ -534,21 +521,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Due Soon</t>
-        </is>
-      </c>
       <c r="C2" s="1" t="n">
-        <v>46138.44337213237</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>46138.51412209345</v>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>b</t>
@@ -560,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.44337213253</v>
+        <v>46138.5141220936</v>
       </c>
     </row>
     <row r="4">
@@ -573,7 +550,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.44337213263</v>
+        <v>46138.51412209368</v>
       </c>
     </row>
     <row r="5">
@@ -586,7 +563,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.44337213269</v>
+        <v>46138.51412209375</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +576,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.44337213277</v>
+        <v>46138.51412209381</v>
       </c>
     </row>
     <row r="7">
@@ -612,7 +589,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.44337213284</v>
+        <v>46138.51412209387</v>
       </c>
     </row>
     <row r="8">
@@ -625,7 +602,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.44337213292</v>
+        <v>46138.51412209393</v>
       </c>
     </row>
     <row r="9">
@@ -638,10 +615,10 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.44337213298</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>46138.51412209399</v>
+      </c>
+    </row>
+    <row r="10" hidden="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>i</t>
@@ -651,7 +628,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.44337213306</v>
+        <v>46138.51412209405</v>
       </c>
     </row>
     <row r="11">
@@ -664,7 +641,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.44337213312</v>
+        <v>46138.51412209411</v>
       </c>
     </row>
     <row r="12">
@@ -686,12 +663,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="7">
+      <c r="B15">
         <f>VLOOKUP("c",A1:C11,2,FALSE)</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -745,7 +725,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46138.44337213237</v>
+        <v>46138.51412209345</v>
       </c>
     </row>
     <row r="3">
@@ -758,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.44337213253</v>
+        <v>46138.5141220936</v>
       </c>
     </row>
     <row r="4">
@@ -771,7 +751,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.44337213263</v>
+        <v>46138.51412209368</v>
       </c>
     </row>
     <row r="5">
@@ -784,7 +764,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.44337213269</v>
+        <v>46138.51412209375</v>
       </c>
     </row>
     <row r="6">
@@ -797,7 +777,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.44337213277</v>
+        <v>46138.51412209381</v>
       </c>
     </row>
     <row r="7">
@@ -810,7 +790,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.44337213284</v>
+        <v>46138.51412209387</v>
       </c>
     </row>
     <row r="8">
@@ -823,7 +803,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.44337213292</v>
+        <v>46138.51412209393</v>
       </c>
     </row>
     <row r="9">
@@ -836,7 +816,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.44337213298</v>
+        <v>46138.51412209399</v>
       </c>
     </row>
     <row r="10">
@@ -849,7 +829,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.44337213306</v>
+        <v>46138.51412209405</v>
       </c>
     </row>
     <row r="11">
@@ -862,7 +842,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.44337213312</v>
+        <v>46138.51412209411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add functionality to freeze panes and print column letters in Excel file manipulation
</commit_message>
<xml_diff>
--- a/Book/chapter14/myExcelFile.xlsx
+++ b/Book/chapter14/myExcelFile.xlsx
@@ -522,7 +522,7 @@
     </row>
     <row r="2">
       <c r="C2" s="1" t="n">
-        <v>46138.51412209345</v>
+        <v>46138.56965036919</v>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.5141220936</v>
+        <v>46138.56965037197</v>
       </c>
     </row>
     <row r="4">
@@ -550,7 +550,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.51412209368</v>
+        <v>46138.56965037461</v>
       </c>
     </row>
     <row r="5">
@@ -563,7 +563,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.51412209375</v>
+        <v>46138.56965037712</v>
       </c>
     </row>
     <row r="6">
@@ -576,7 +576,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.51412209381</v>
+        <v>46138.5696503797</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.51412209387</v>
+        <v>46138.56965038217</v>
       </c>
     </row>
     <row r="8">
@@ -602,7 +602,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.51412209393</v>
+        <v>46138.56965038474</v>
       </c>
     </row>
     <row r="9">
@@ -615,7 +615,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.51412209399</v>
+        <v>46138.56965038725</v>
       </c>
     </row>
     <row r="10" hidden="1">
@@ -628,7 +628,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.51412209405</v>
+        <v>46138.5696503898</v>
       </c>
     </row>
     <row r="11">
@@ -641,7 +641,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.51412209411</v>
+        <v>46138.56965039238</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46138.51412209345</v>
+        <v>46138.56965036919</v>
       </c>
     </row>
     <row r="3">
@@ -738,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46138.5141220936</v>
+        <v>46138.56965037197</v>
       </c>
     </row>
     <row r="4">
@@ -751,7 +751,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46138.51412209368</v>
+        <v>46138.56965037461</v>
       </c>
     </row>
     <row r="5">
@@ -764,7 +764,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46138.51412209375</v>
+        <v>46138.56965037712</v>
       </c>
     </row>
     <row r="6">
@@ -777,7 +777,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46138.51412209381</v>
+        <v>46138.5696503797</v>
       </c>
     </row>
     <row r="7">
@@ -790,7 +790,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46138.51412209387</v>
+        <v>46138.56965038217</v>
       </c>
     </row>
     <row r="8">
@@ -803,7 +803,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46138.51412209393</v>
+        <v>46138.56965038474</v>
       </c>
     </row>
     <row r="9">
@@ -816,7 +816,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46138.51412209399</v>
+        <v>46138.56965038725</v>
       </c>
     </row>
     <row r="10">
@@ -829,7 +829,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46138.51412209405</v>
+        <v>46138.5696503898</v>
       </c>
     </row>
     <row r="11">
@@ -842,7 +842,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46138.51412209411</v>
+        <v>46138.56965039238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>